<commit_message>
update: public/quintessential-essence/3 Cloudfarms/Samlet Rapport.md public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx scripts/navigationData.generated.js
</commit_message>
<xml_diff>
--- a/public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx
+++ b/public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx
@@ -519,7 +519,7 @@
         <v>89</v>
       </c>
       <c r="P3" t="str">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
@@ -569,7 +569,7 @@
         <v>7.87</v>
       </c>
       <c r="P4" t="str">
-        <v>3.57</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         <v>5.6</v>
       </c>
       <c r="P5" t="str">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="6">
@@ -1624,7 +1624,7 @@
         <v>17.7</v>
       </c>
       <c r="P27" t="str">
-        <v>7.4</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="28">
@@ -1674,7 +1674,7 @@
         <v>2.17</v>
       </c>
       <c r="P28" t="str">
-        <v>2.3</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="29">
@@ -1724,7 +1724,7 @@
         <v>41</v>
       </c>
       <c r="P29" t="str">
-        <v>44.2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
update: "convert vacxin/Output/2 Vaccination af s\303\270er 4 uger f\303\270r faring/Vaccination_Rapport.md" convert vacxin/service-list-10.xlsx convert vacxin/service-list-11.xlsx convert vacxin/service-list-12.xlsx convert vacxin/service-list-13.xlsx convert vacxin/service-list-14.xlsx convert vacxin/service-list-6.xlsx convert vacxin/service-list-7.xlsx convert vacxin/service-list-8.xlsx convert vacxin/service-list-9.xlsx convert/coudfarms/Input/07 2026.xlsx convert/coudfarms/Input/production-report(6).xlsx public/quintessential-essence/3 Cloudfarms/Samlet Rapport.md public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx
</commit_message>
<xml_diff>
--- a/public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx
+++ b/public/quintessential-essence/3 Cloudfarms/Samlet Rapport.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:Q31"/>
   <cols>
     <col min="1" max="1" width="45.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -415,6 +415,7 @@
     <col min="14" max="14" width="10.83203125" customWidth="1"/>
     <col min="15" max="15" width="10.83203125" customWidth="1"/>
     <col min="16" max="16" width="10.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,27 +449,30 @@
         <v>Tuần 6</v>
       </c>
       <c r="I2" t="str">
+        <v>Tuần 7</v>
+      </c>
+      <c r="J2" t="str">
         <v>Tuần 8</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Tuần 9</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Tuần 10</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Tuần 11</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Tuần 12</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>Tuần 13</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>Tuần 14</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>Tuần 15</v>
       </c>
     </row>
@@ -498,27 +502,30 @@
         <v>88</v>
       </c>
       <c r="I3" t="str">
+        <v>89</v>
+      </c>
+      <c r="J3" t="str">
         <v>88</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>90</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>88</v>
-      </c>
-      <c r="L3" t="str">
-        <v>91</v>
       </c>
       <c r="M3" t="str">
         <v>91</v>
       </c>
       <c r="N3" t="str">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O3" t="str">
         <v>89</v>
       </c>
       <c r="P3" t="str">
+        <v>89</v>
+      </c>
+      <c r="Q3" t="str">
         <v>90</v>
       </c>
     </row>
@@ -548,27 +555,30 @@
         <v>2.27</v>
       </c>
       <c r="I4" t="str">
+        <v>2.25</v>
+      </c>
+      <c r="J4" t="str">
         <v>5.68</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>4.44</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>3.41</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>2.2</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>7.69</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>2.25</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>7.87</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>4.44</v>
       </c>
     </row>
@@ -598,27 +608,30 @@
         <v>5.7</v>
       </c>
       <c r="I5" t="str">
+        <v>6.9</v>
+      </c>
+      <c r="J5" t="str">
         <v>8.2</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>6.7</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>6.8</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>6.3</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>6.9</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>7.1</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>5.6</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v>5.4</v>
       </c>
     </row>
@@ -648,27 +661,30 @@
         <v>93.3</v>
       </c>
       <c r="I6" t="str">
+        <v>98.9</v>
+      </c>
+      <c r="J6" t="str">
         <v>96.6</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>98.9</v>
-      </c>
-      <c r="K6" t="str">
-        <v>96.6</v>
       </c>
       <c r="L6" t="str">
         <v>96.6</v>
       </c>
       <c r="M6" t="str">
+        <v>96.6</v>
+      </c>
+      <c r="N6" t="str">
         <v>98.9</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>95.6</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>94.3</v>
       </c>
-      <c r="P6" t="str">
+      <c r="Q6" t="str">
         <v>96.7</v>
       </c>
     </row>
@@ -698,27 +714,30 @@
         <v>96.6</v>
       </c>
       <c r="I7" t="str">
+        <v>93.3</v>
+      </c>
+      <c r="J7" t="str">
         <v>91.1</v>
-      </c>
-      <c r="J7" t="str">
-        <v>94.4</v>
       </c>
       <c r="K7" t="str">
         <v>94.4</v>
       </c>
       <c r="L7" t="str">
+        <v>94.4</v>
+      </c>
+      <c r="M7" t="str">
         <v>94.3</v>
       </c>
-      <c r="M7" t="str">
+      <c r="N7" t="str">
         <v>93.2</v>
       </c>
-      <c r="N7" t="str">
+      <c r="O7" t="str">
         <v>88.8</v>
       </c>
-      <c r="O7" t="str">
+      <c r="P7" t="str">
         <v>97.7</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v>94.4</v>
       </c>
     </row>
@@ -748,27 +767,30 @@
         <v>92.2</v>
       </c>
       <c r="I8" t="str">
+        <v>91.2</v>
+      </c>
+      <c r="J8" t="str">
         <v>95.5</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>92.1</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>90</v>
       </c>
-      <c r="L8" t="str">
+      <c r="M8" t="str">
         <v>94.4</v>
       </c>
-      <c r="M8" t="str">
+      <c r="N8" t="str">
         <v>92.1</v>
       </c>
-      <c r="N8" t="str">
+      <c r="O8" t="str">
         <v>93.1</v>
       </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
         <v>90.9</v>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>86.5</v>
       </c>
     </row>
@@ -798,19 +820,19 @@
         <v>11</v>
       </c>
       <c r="I9" t="str">
+        <v>7</v>
+      </c>
+      <c r="J9" t="str">
         <v>8</v>
       </c>
-      <c r="J9" t="str">
+      <c r="K9" t="str">
         <v>7</v>
-      </c>
-      <c r="K9" t="str">
-        <v>4</v>
       </c>
       <c r="L9" t="str">
         <v>4</v>
       </c>
       <c r="M9" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" t="str">
         <v>3</v>
@@ -819,6 +841,9 @@
         <v>3</v>
       </c>
       <c r="P9" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="str">
         <v>5</v>
       </c>
     </row>
@@ -853,27 +878,30 @@
         <v>Tuần 6</v>
       </c>
       <c r="I12" t="str">
+        <v>Tuần 7</v>
+      </c>
+      <c r="J12" t="str">
         <v>Tuần 8</v>
       </c>
-      <c r="J12" t="str">
+      <c r="K12" t="str">
         <v>Tuần 9</v>
       </c>
-      <c r="K12" t="str">
+      <c r="L12" t="str">
         <v>Tuần 10</v>
       </c>
-      <c r="L12" t="str">
+      <c r="M12" t="str">
         <v>Tuần 11</v>
       </c>
-      <c r="M12" t="str">
+      <c r="N12" t="str">
         <v>Tuần 12</v>
       </c>
-      <c r="N12" t="str">
+      <c r="O12" t="str">
         <v>Tuần 13</v>
       </c>
-      <c r="O12" t="str">
+      <c r="P12" t="str">
         <v>Tuần 14</v>
       </c>
-      <c r="P12" t="str">
+      <c r="Q12" t="str">
         <v>Tuần 15</v>
       </c>
     </row>
@@ -903,27 +931,30 @@
         <v>81</v>
       </c>
       <c r="I13" t="str">
+        <v>86</v>
+      </c>
+      <c r="J13" t="str">
         <v>73</v>
       </c>
-      <c r="J13" t="str">
+      <c r="K13" t="str">
         <v>82</v>
       </c>
-      <c r="K13" t="str">
+      <c r="L13" t="str">
         <v>77</v>
       </c>
-      <c r="L13" t="str">
+      <c r="M13" t="str">
         <v>81</v>
       </c>
-      <c r="M13" t="str">
+      <c r="N13" t="str">
         <v>72</v>
       </c>
-      <c r="N13" t="str">
+      <c r="O13" t="str">
         <v>83</v>
       </c>
-      <c r="O13" t="str">
+      <c r="P13" t="str">
         <v>77</v>
       </c>
-      <c r="P13" t="str">
+      <c r="Q13" t="str">
         <v>84</v>
       </c>
     </row>
@@ -953,27 +984,30 @@
         <v>91.2</v>
       </c>
       <c r="I14" t="str">
+        <v>91.3</v>
+      </c>
+      <c r="J14" t="str">
         <v>82.6</v>
       </c>
-      <c r="J14" t="str">
+      <c r="K14" t="str">
         <v>88</v>
       </c>
-      <c r="K14" t="str">
+      <c r="L14" t="str">
         <v>87.6</v>
       </c>
-      <c r="L14" t="str">
+      <c r="M14" t="str">
         <v>86.7</v>
       </c>
-      <c r="M14" t="str">
+      <c r="N14" t="str">
         <v>82.6</v>
       </c>
-      <c r="N14" t="str">
+      <c r="O14" t="str">
         <v>93.3</v>
       </c>
-      <c r="O14" t="str">
+      <c r="P14" t="str">
         <v>87.8</v>
       </c>
-      <c r="P14" t="str">
+      <c r="Q14" t="str">
         <v>91.1</v>
       </c>
     </row>
@@ -1003,27 +1037,30 @@
         <v>19.8</v>
       </c>
       <c r="I15" t="str">
+        <v>20.5</v>
+      </c>
+      <c r="J15" t="str">
         <v>19.7</v>
       </c>
-      <c r="J15" t="str">
+      <c r="K15" t="str">
         <v>20</v>
       </c>
-      <c r="K15" t="str">
+      <c r="L15" t="str">
         <v>20.4</v>
       </c>
-      <c r="L15" t="str">
+      <c r="M15" t="str">
         <v>20.2</v>
       </c>
-      <c r="M15" t="str">
+      <c r="N15" t="str">
         <v>19.9</v>
       </c>
-      <c r="N15" t="str">
+      <c r="O15" t="str">
         <v>20.6</v>
       </c>
-      <c r="O15" t="str">
+      <c r="P15" t="str">
         <v>21</v>
       </c>
-      <c r="P15" t="str">
+      <c r="Q15" t="str">
         <v>21.1</v>
       </c>
     </row>
@@ -1053,27 +1090,30 @@
         <v>18.7</v>
       </c>
       <c r="I16" t="str">
+        <v>18.2</v>
+      </c>
+      <c r="J16" t="str">
         <v>17.9</v>
       </c>
-      <c r="J16" t="str">
+      <c r="K16" t="str">
         <v>16.5</v>
       </c>
-      <c r="K16" t="str">
+      <c r="L16" t="str">
         <v>17.4</v>
       </c>
-      <c r="L16" t="str">
+      <c r="M16" t="str">
         <v>17</v>
       </c>
-      <c r="M16" t="str">
+      <c r="N16" t="str">
         <v>17.4</v>
       </c>
-      <c r="N16" t="str">
+      <c r="O16" t="str">
         <v>17.5</v>
       </c>
-      <c r="O16" t="str">
+      <c r="P16" t="str">
         <v>18.6</v>
       </c>
-      <c r="P16" t="str">
+      <c r="Q16" t="str">
         <v>19.1</v>
       </c>
     </row>
@@ -1103,27 +1143,30 @@
         <v>1.3</v>
       </c>
       <c r="I17" t="str">
+        <v>1.2</v>
+      </c>
+      <c r="J17" t="str">
         <v>1.6</v>
       </c>
-      <c r="J17" t="str">
+      <c r="K17" t="str">
         <v>1.3</v>
       </c>
-      <c r="K17" t="str">
+      <c r="L17" t="str">
         <v>1.4</v>
       </c>
-      <c r="L17" t="str">
+      <c r="M17" t="str">
         <v>1.5</v>
       </c>
-      <c r="M17" t="str">
+      <c r="N17" t="str">
         <v>1.3</v>
       </c>
-      <c r="N17" t="str">
+      <c r="O17" t="str">
         <v>1.4</v>
       </c>
-      <c r="O17" t="str">
+      <c r="P17" t="str">
         <v>1.2</v>
       </c>
-      <c r="P17" t="str">
+      <c r="Q17" t="str">
         <v>1.2</v>
       </c>
     </row>
@@ -1153,27 +1196,30 @@
         <v>197</v>
       </c>
       <c r="I18" t="str">
+        <v>213</v>
+      </c>
+      <c r="J18" t="str">
         <v>173</v>
       </c>
-      <c r="J18" t="str">
+      <c r="K18" t="str">
         <v>202</v>
       </c>
-      <c r="K18" t="str">
+      <c r="L18" t="str">
         <v>184</v>
       </c>
-      <c r="L18" t="str">
+      <c r="M18" t="str">
         <v>246</v>
       </c>
-      <c r="M18" t="str">
+      <c r="N18" t="str">
         <v>153</v>
       </c>
-      <c r="N18" t="str">
+      <c r="O18" t="str">
         <v>189</v>
       </c>
-      <c r="O18" t="str">
+      <c r="P18" t="str">
         <v>177</v>
       </c>
-      <c r="P18" t="str">
+      <c r="Q18" t="str">
         <v>121</v>
       </c>
     </row>
@@ -1203,27 +1249,30 @@
         <v>12.26</v>
       </c>
       <c r="I19" t="str">
+        <v>12.07</v>
+      </c>
+      <c r="J19" t="str">
         <v>12.01</v>
       </c>
-      <c r="J19" t="str">
+      <c r="K19" t="str">
         <v>12.29</v>
       </c>
-      <c r="K19" t="str">
+      <c r="L19" t="str">
         <v>11.71</v>
       </c>
-      <c r="L19" t="str">
+      <c r="M19" t="str">
         <v>15</v>
       </c>
-      <c r="M19" t="str">
+      <c r="N19" t="str">
         <v>10.68</v>
       </c>
-      <c r="N19" t="str">
+      <c r="O19" t="str">
         <v>11.03</v>
       </c>
-      <c r="O19" t="str">
+      <c r="P19" t="str">
         <v>10.93</v>
       </c>
-      <c r="P19" t="str">
+      <c r="Q19" t="str">
         <v>6.83</v>
       </c>
     </row>
@@ -1253,27 +1302,30 @@
         <v>117</v>
       </c>
       <c r="I20" t="str">
+        <v>122</v>
+      </c>
+      <c r="J20" t="str">
         <v>103</v>
       </c>
-      <c r="J20" t="str">
+      <c r="K20" t="str">
         <v>127</v>
       </c>
-      <c r="K20" t="str">
+      <c r="L20" t="str">
         <v>123</v>
       </c>
-      <c r="L20" t="str">
+      <c r="M20" t="str">
         <v>120</v>
       </c>
-      <c r="M20" t="str">
+      <c r="N20" t="str">
         <v>110</v>
       </c>
-      <c r="N20" t="str">
+      <c r="O20" t="str">
         <v>121</v>
       </c>
-      <c r="O20" t="str">
+      <c r="P20" t="str">
         <v>113</v>
       </c>
-      <c r="P20" t="str">
+      <c r="Q20" t="str">
         <v>119</v>
       </c>
     </row>
@@ -1303,27 +1355,30 @@
         <v>1404</v>
       </c>
       <c r="I21" t="str">
+        <v>1479</v>
+      </c>
+      <c r="J21" t="str">
         <v>1231</v>
       </c>
-      <c r="J21" t="str">
+      <c r="K21" t="str">
         <v>1513</v>
       </c>
-      <c r="K21" t="str">
+      <c r="L21" t="str">
         <v>1488</v>
       </c>
-      <c r="L21" t="str">
+      <c r="M21" t="str">
         <v>1415</v>
       </c>
-      <c r="M21" t="str">
+      <c r="N21" t="str">
         <v>1280</v>
       </c>
-      <c r="N21" t="str">
+      <c r="O21" t="str">
         <v>1468</v>
       </c>
-      <c r="O21" t="str">
+      <c r="P21" t="str">
         <v>1358</v>
       </c>
-      <c r="P21" t="str">
+      <c r="Q21" t="str">
         <v>1477</v>
       </c>
     </row>
@@ -1353,27 +1408,30 @@
         <v>12</v>
       </c>
       <c r="I22" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="J22" t="str">
         <v>12</v>
       </c>
-      <c r="J22" t="str">
+      <c r="K22" t="str">
         <v>11.9</v>
       </c>
-      <c r="K22" t="str">
+      <c r="L22" t="str">
         <v>12.1</v>
       </c>
-      <c r="L22" t="str">
+      <c r="M22" t="str">
         <v>11.8</v>
       </c>
-      <c r="M22" t="str">
+      <c r="N22" t="str">
         <v>11.6</v>
       </c>
-      <c r="N22" t="str">
+      <c r="O22" t="str">
         <v>12.1</v>
       </c>
-      <c r="O22" t="str">
+      <c r="P22" t="str">
         <v>12</v>
       </c>
-      <c r="P22" t="str">
+      <c r="Q22" t="str">
         <v>12.4</v>
       </c>
     </row>
@@ -1403,27 +1461,30 @@
         <v>16.9</v>
       </c>
       <c r="I23" t="str">
+        <v>19.2</v>
+      </c>
+      <c r="J23" t="str">
         <v>17.3</v>
       </c>
-      <c r="J23" t="str">
+      <c r="K23" t="str">
         <v>18.5</v>
       </c>
-      <c r="K23" t="str">
+      <c r="L23" t="str">
         <v>17.5</v>
       </c>
-      <c r="L23" t="str">
+      <c r="M23" t="str">
         <v>17</v>
       </c>
-      <c r="M23" t="str">
+      <c r="N23" t="str">
         <v>16.6</v>
       </c>
-      <c r="N23" t="str">
+      <c r="O23" t="str">
         <v>18.8</v>
       </c>
-      <c r="O23" t="str">
+      <c r="P23" t="str">
         <v>18.9</v>
       </c>
-      <c r="P23" t="str">
+      <c r="Q23" t="str">
         <v>19.2</v>
       </c>
     </row>
@@ -1453,27 +1514,30 @@
         <v>27.3</v>
       </c>
       <c r="I24" t="str">
+        <v>12.6</v>
+      </c>
+      <c r="J24" t="str">
         <v>12.3</v>
       </c>
-      <c r="J24" t="str">
+      <c r="K24" t="str">
         <v>11.8</v>
       </c>
-      <c r="K24" t="str">
+      <c r="L24" t="str">
         <v>9</v>
       </c>
-      <c r="L24" t="str">
+      <c r="M24" t="str">
         <v>13.2</v>
       </c>
-      <c r="M24" t="str">
+      <c r="N24" t="str">
         <v>17.9</v>
       </c>
-      <c r="N24" t="str">
+      <c r="O24" t="str">
         <v>18.9</v>
       </c>
-      <c r="O24" t="str">
+      <c r="P24" t="str">
         <v>11.1</v>
       </c>
-      <c r="P24" t="str">
+      <c r="Q24" t="str">
         <v>-4.5</v>
       </c>
     </row>
@@ -1506,24 +1570,27 @@
         <v>29</v>
       </c>
       <c r="J25" t="str">
+        <v>29</v>
+      </c>
+      <c r="K25" t="str">
         <v>30</v>
       </c>
-      <c r="K25" t="str">
+      <c r="L25" t="str">
         <v>31</v>
       </c>
-      <c r="L25" t="str">
+      <c r="M25" t="str">
         <v>30</v>
       </c>
-      <c r="M25" t="str">
+      <c r="N25" t="str">
         <v>31</v>
       </c>
-      <c r="N25" t="str">
+      <c r="O25" t="str">
         <v>30</v>
       </c>
-      <c r="O25" t="str">
+      <c r="P25" t="str">
         <v>32</v>
       </c>
-      <c r="P25" t="str">
+      <c r="Q25" t="str">
         <v>32</v>
       </c>
     </row>
@@ -1559,7 +1626,7 @@
         <v>118</v>
       </c>
       <c r="K26" t="str">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L26" t="str">
         <v>119</v>
@@ -1571,9 +1638,12 @@
         <v>119</v>
       </c>
       <c r="O26" t="str">
+        <v>119</v>
+      </c>
+      <c r="P26" t="str">
         <v>118</v>
       </c>
-      <c r="P26" t="str">
+      <c r="Q26" t="str">
         <v>119</v>
       </c>
     </row>
@@ -1603,27 +1673,30 @@
         <v>17.2</v>
       </c>
       <c r="I27" t="str">
+        <v>15.5</v>
+      </c>
+      <c r="J27" t="str">
         <v>20.4</v>
       </c>
-      <c r="J27" t="str">
+      <c r="K27" t="str">
         <v>12.9</v>
       </c>
-      <c r="K27" t="str">
+      <c r="L27" t="str">
         <v>12.8</v>
       </c>
-      <c r="L27" t="str">
+      <c r="M27" t="str">
         <v>10</v>
       </c>
-      <c r="M27" t="str">
+      <c r="N27" t="str">
         <v>15.1</v>
       </c>
-      <c r="N27" t="str">
+      <c r="O27" t="str">
         <v>10.4</v>
       </c>
-      <c r="O27" t="str">
+      <c r="P27" t="str">
         <v>17.7</v>
       </c>
-      <c r="P27" t="str">
+      <c r="Q27" t="str">
         <v>8.1</v>
       </c>
     </row>
@@ -1653,27 +1726,30 @@
         <v>2.22</v>
       </c>
       <c r="I28" t="str">
+        <v>2.24</v>
+      </c>
+      <c r="J28" t="str">
         <v>2.17</v>
       </c>
-      <c r="J28" t="str">
+      <c r="K28" t="str">
         <v>2.26</v>
       </c>
-      <c r="K28" t="str">
+      <c r="L28" t="str">
         <v>2.25</v>
       </c>
-      <c r="L28" t="str">
+      <c r="M28" t="str">
         <v>2.31</v>
       </c>
-      <c r="M28" t="str">
+      <c r="N28" t="str">
         <v>2.22</v>
       </c>
-      <c r="N28" t="str">
+      <c r="O28" t="str">
         <v>2.3</v>
       </c>
-      <c r="O28" t="str">
+      <c r="P28" t="str">
         <v>2.17</v>
       </c>
-      <c r="P28" t="str">
+      <c r="Q28" t="str">
         <v>2.29</v>
       </c>
     </row>
@@ -1703,27 +1779,30 @@
         <v>37.6</v>
       </c>
       <c r="I29" t="str">
+        <v>43</v>
+      </c>
+      <c r="J29" t="str">
         <v>37.6</v>
       </c>
-      <c r="J29" t="str">
+      <c r="K29" t="str">
         <v>41.7</v>
-      </c>
-      <c r="K29" t="str">
-        <v>39.3</v>
       </c>
       <c r="L29" t="str">
         <v>39.3</v>
       </c>
       <c r="M29" t="str">
+        <v>39.3</v>
+      </c>
+      <c r="N29" t="str">
         <v>36.9</v>
       </c>
-      <c r="N29" t="str">
+      <c r="O29" t="str">
         <v>43.3</v>
       </c>
-      <c r="O29" t="str">
+      <c r="P29" t="str">
         <v>41</v>
       </c>
-      <c r="P29" t="str">
+      <c r="Q29" t="str">
         <v>44</v>
       </c>
     </row>
@@ -1753,27 +1832,30 @@
         <v>39.1</v>
       </c>
       <c r="I30" t="str">
+        <v>41.4</v>
+      </c>
+      <c r="J30" t="str">
         <v>34.6</v>
       </c>
-      <c r="J30" t="str">
+      <c r="K30" t="str">
         <v>42.6</v>
       </c>
-      <c r="K30" t="str">
+      <c r="L30" t="str">
         <v>41.8</v>
       </c>
-      <c r="L30" t="str">
+      <c r="M30" t="str">
         <v>39.5</v>
       </c>
-      <c r="M30" t="str">
+      <c r="N30" t="str">
         <v>36.1</v>
       </c>
-      <c r="N30" t="str">
+      <c r="O30" t="str">
         <v>41.5</v>
       </c>
-      <c r="O30" t="str">
+      <c r="P30" t="str">
         <v>38.4</v>
       </c>
-      <c r="P30" t="str">
+      <c r="Q30" t="str">
         <v>43.1</v>
       </c>
     </row>
@@ -1803,33 +1885,36 @@
         <v>183</v>
       </c>
       <c r="I31" t="str">
+        <v>193</v>
+      </c>
+      <c r="J31" t="str">
         <v>161</v>
       </c>
-      <c r="J31" t="str">
+      <c r="K31" t="str">
         <v>198</v>
       </c>
-      <c r="K31" t="str">
+      <c r="L31" t="str">
         <v>194</v>
       </c>
-      <c r="L31" t="str">
+      <c r="M31" t="str">
         <v>183</v>
       </c>
-      <c r="M31" t="str">
+      <c r="N31" t="str">
         <v>167</v>
       </c>
-      <c r="N31" t="str">
+      <c r="O31" t="str">
         <v>192</v>
       </c>
-      <c r="O31" t="str">
+      <c r="P31" t="str">
         <v>177</v>
       </c>
-      <c r="P31" t="str">
+      <c r="Q31" t="str">
         <v>199</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>